<commit_message>
Add new manually labeled datasets and code for impacted titles/sectors plots
</commit_message>
<xml_diff>
--- a/data/manually_labeled/work_related_100.xlsx
+++ b/data/manually_labeled/work_related_100.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriele/Documents/progetti_politecnico/chatgpt-at-work/chatgpt-at-work/data/manually_labeled/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69D0105-51FA-FD4D-AEA5-E7CB95ACA73E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7898856B-6279-3D45-83CB-9011FFC019CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="106">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -6553,6 +6553,9 @@
       <c r="C32" t="s">
         <v>6</v>
       </c>
+      <c r="D32" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="33" spans="1:4" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A33">

</xml_diff>